<commit_message>
SSHv1.4 - Excel export hata duzeltmeleri ve FAB pozisyon
- FIX: ExcelReportGenerator NameError (service_status.py L707,L734) -> AvailabilityExcelGenerator import
- FIX: hbr_download path traversal -> secure_filename() eklendi
- FIX: Path traversal korunmasi (service_status.py comprehensive/root-cause/daily)
- FIX: tram_id DB dogrulamasi (daily report)
- FIX: Bos arac listesi kontrolu (5 fonksiyon)
- FIX: Bare except:pass -> except (ValueError, TypeError) (kpi.py, fracas.py)
- FIX: Temp dosya temizligi after_this_request ile (ariza export)
- FAB buton sag uste tasindi

4 dosya, 71 ekleme, 33 silme
</commit_message>
<xml_diff>
--- a/data/kayseri/km_data.xlsx
+++ b/data/kayseri/km_data.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>218955</v>
+        <v>227108</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-02 14:23:21</t>
+          <t>2026-03-31 14:42:33</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>usahin</t>
         </is>
       </c>
     </row>
@@ -470,16 +470,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>206632</v>
+        <v>214749</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-02 14:23:21</t>
+          <t>2026-03-31 14:42:33</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>usahin</t>
         </is>
       </c>
     </row>
@@ -490,16 +490,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>170334</v>
+        <v>176943</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-03-02 14:23:22</t>
+          <t>2026-03-31 14:42:33</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>usahin</t>
         </is>
       </c>
     </row>
@@ -510,16 +510,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>218289</v>
+        <v>219968</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-02 14:23:22</t>
+          <t>2026-03-31 14:42:33</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>usahin</t>
         </is>
       </c>
     </row>
@@ -530,16 +530,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>142614</v>
+        <v>149779</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-02 14:23:22</t>
+          <t>2026-03-31 14:42:34</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>usahin</t>
         </is>
       </c>
     </row>
@@ -550,16 +550,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>184781</v>
+        <v>188930</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-03-02 14:23:22</t>
+          <t>2026-03-31 14:42:34</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>usahin</t>
         </is>
       </c>
     </row>
@@ -570,16 +570,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>176687</v>
+        <v>185311</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-03-02 14:23:22</t>
+          <t>2026-03-31 14:42:34</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>usahin</t>
         </is>
       </c>
     </row>
@@ -590,16 +590,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>154363</v>
+        <v>161082</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-03-02 14:23:22</t>
+          <t>2026-03-31 14:42:34</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>usahin</t>
         </is>
       </c>
     </row>
@@ -610,16 +610,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>161453</v>
+        <v>170005</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-03-02 14:23:22</t>
+          <t>2026-03-31 14:42:35</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>usahin</t>
         </is>
       </c>
     </row>
@@ -630,17 +630,37 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>158676</v>
+        <v>162151</v>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-02 14:23:22</t>
+          <t>2026-03-31 14:42:35</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>usahin</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>3872</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>200383</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-03-31 14:42:32</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>usahin</t>
         </is>
       </c>
     </row>

</xml_diff>